<commit_message>
fixed arni dose text in var desc
</commit_message>
<xml_diff>
--- a/docs/variabledescription/meta_variables.xlsx
+++ b/docs/variabledescription/meta_variables.xlsx
@@ -8,17 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\k2_stat_heartfailure\Projects\20240619_shfdb5\dm\metadata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9560219B-D901-4F03-8F15-435947D783C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9EA85F3-D00B-497B-B15C-7F6BDC97139C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId2"/>
-  </externalReferences>
-  <calcPr calcId="0" concurrentCalc="0"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
@@ -1629,22 +1626,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
-      <sheetName val="Sheet 1"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3609,7 +3590,7 @@
         <v>494</v>
       </c>
       <c r="B142" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="C142" t="s">
         <v>201</v>
@@ -3637,7 +3618,7 @@
         <v>496</v>
       </c>
       <c r="B144" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="C144" t="s">
         <v>201</v>

</xml_diff>

<commit_message>
v 502 added ef dtm
</commit_message>
<xml_diff>
--- a/docs/variabledescription/meta_variables.xlsx
+++ b/docs/variabledescription/meta_variables.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\k2_stat_heartfailure\Projects\20240619_shfdb5\dm\metadata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D39DDA5B-1A27-4747-933F-E475C9629870}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77A4CA0D-3A31-4BBB-8ADF-86CD3D41E768}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="755" uniqueCount="506">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="757" uniqueCount="508">
   <si>
     <t>lopnr</t>
   </si>
@@ -1538,6 +1538,12 @@
   </si>
   <si>
     <t>ICD-codes see https://kiheartfailure.github.io/shfdb5/definitions/. Also see shf_af</t>
+  </si>
+  <si>
+    <t>Date of LVEF</t>
+  </si>
+  <si>
+    <t>shf_efdtm</t>
   </si>
 </sst>
 </file>
@@ -1907,7 +1913,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E239"/>
+  <dimension ref="A1:E240"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="33.140625" customWidth="1"/>
@@ -2075,26 +2081,23 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>10</v>
+        <v>507</v>
       </c>
       <c r="B15" t="s">
-        <v>205</v>
+        <v>506</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B16" t="s">
-        <v>206</v>
-      </c>
-      <c r="C16" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>93</v>
+        <v>11</v>
       </c>
       <c r="B17" t="s">
         <v>206</v>
@@ -2105,72 +2108,75 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>12</v>
+        <v>93</v>
       </c>
       <c r="B18" t="s">
-        <v>208</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>209</v>
+        <v>206</v>
+      </c>
+      <c r="C18" t="s">
+        <v>207</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B19" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B20" t="s">
-        <v>213</v>
-      </c>
-      <c r="E20" t="s">
-        <v>214</v>
+        <v>211</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>212</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B21" t="s">
-        <v>215</v>
+        <v>213</v>
+      </c>
+      <c r="E21" t="s">
+        <v>214</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B22" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B23" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B24" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>94</v>
+        <v>18</v>
       </c>
       <c r="B25" t="s">
         <v>218</v>
@@ -2178,51 +2184,51 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>19</v>
+        <v>94</v>
       </c>
       <c r="B26" t="s">
-        <v>371</v>
+        <v>218</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B27" t="s">
-        <v>219</v>
-      </c>
-      <c r="C27" t="s">
-        <v>461</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>220</v>
-      </c>
-      <c r="E27" t="s">
-        <v>221</v>
+        <v>371</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B28" t="s">
-        <v>222</v>
+        <v>219</v>
+      </c>
+      <c r="C28" t="s">
+        <v>461</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>223</v>
+        <v>220</v>
+      </c>
+      <c r="E28" t="s">
+        <v>221</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B29" t="s">
-        <v>224</v>
+        <v>222</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>223</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>92</v>
+        <v>22</v>
       </c>
       <c r="B30" t="s">
         <v>224</v>
@@ -2230,49 +2236,43 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>23</v>
+        <v>92</v>
       </c>
       <c r="B31" t="s">
-        <v>372</v>
-      </c>
-      <c r="D31" s="2" t="s">
-        <v>202</v>
+        <v>224</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B32" t="s">
-        <v>225</v>
-      </c>
-      <c r="C32" t="s">
-        <v>226</v>
-      </c>
-      <c r="E32" t="s">
-        <v>430</v>
+        <v>372</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>202</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>427</v>
+        <v>24</v>
       </c>
       <c r="B33" t="s">
-        <v>443</v>
+        <v>225</v>
       </c>
       <c r="C33" t="s">
         <v>226</v>
       </c>
-      <c r="D33" s="2" t="s">
-        <v>202</v>
+      <c r="E33" t="s">
+        <v>430</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="B34" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="C34" t="s">
         <v>226</v>
@@ -2283,52 +2283,52 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>25</v>
+        <v>426</v>
       </c>
       <c r="B35" t="s">
-        <v>227</v>
+        <v>444</v>
       </c>
       <c r="C35" t="s">
-        <v>228</v>
-      </c>
-      <c r="E35" t="s">
-        <v>229</v>
+        <v>226</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>202</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B36" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="C36" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="E36" t="s">
-        <v>430</v>
+        <v>229</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>428</v>
+        <v>26</v>
       </c>
       <c r="B37" t="s">
-        <v>453</v>
+        <v>230</v>
       </c>
       <c r="C37" t="s">
         <v>231</v>
       </c>
-      <c r="D37" s="2" t="s">
-        <v>202</v>
+      <c r="E37" t="s">
+        <v>430</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>425</v>
+        <v>428</v>
       </c>
       <c r="B38" t="s">
-        <v>445</v>
+        <v>453</v>
       </c>
       <c r="C38" t="s">
         <v>231</v>
@@ -2337,40 +2337,40 @@
         <v>202</v>
       </c>
     </row>
-    <row r="39" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>27</v>
+        <v>425</v>
       </c>
       <c r="B39" t="s">
-        <v>232</v>
+        <v>445</v>
       </c>
       <c r="C39" t="s">
         <v>231</v>
       </c>
-      <c r="E39" t="s">
-        <v>430</v>
+      <c r="D39" s="2" t="s">
+        <v>202</v>
       </c>
     </row>
     <row r="40" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>429</v>
+        <v>27</v>
       </c>
       <c r="B40" t="s">
-        <v>454</v>
+        <v>232</v>
       </c>
       <c r="C40" t="s">
         <v>231</v>
       </c>
-      <c r="D40" s="2" t="s">
-        <v>202</v>
+      <c r="E40" t="s">
+        <v>430</v>
       </c>
     </row>
     <row r="41" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>424</v>
+        <v>429</v>
       </c>
       <c r="B41" t="s">
-        <v>446</v>
+        <v>454</v>
       </c>
       <c r="C41" t="s">
         <v>231</v>
@@ -2379,20 +2379,23 @@
         <v>202</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>28</v>
+        <v>424</v>
       </c>
       <c r="B42" t="s">
-        <v>233</v>
+        <v>446</v>
       </c>
       <c r="C42" t="s">
         <v>231</v>
       </c>
+      <c r="D42" s="2" t="s">
+        <v>202</v>
+      </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>96</v>
+        <v>28</v>
       </c>
       <c r="B43" t="s">
         <v>233</v>
@@ -2403,21 +2406,18 @@
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>29</v>
+        <v>96</v>
       </c>
       <c r="B44" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C44" t="s">
-        <v>235</v>
-      </c>
-      <c r="E44" t="s">
-        <v>430</v>
+        <v>231</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>98</v>
+        <v>29</v>
       </c>
       <c r="B45" t="s">
         <v>234</v>
@@ -2425,27 +2425,27 @@
       <c r="C45" t="s">
         <v>235</v>
       </c>
+      <c r="E45" t="s">
+        <v>430</v>
+      </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>436</v>
+        <v>98</v>
       </c>
       <c r="B46" t="s">
-        <v>455</v>
+        <v>234</v>
       </c>
       <c r="C46" t="s">
         <v>235</v>
       </c>
-      <c r="D46" s="2" t="s">
-        <v>202</v>
-      </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>431</v>
+        <v>436</v>
       </c>
       <c r="B47" t="s">
-        <v>447</v>
+        <v>455</v>
       </c>
       <c r="C47" t="s">
         <v>235</v>
@@ -2456,38 +2456,38 @@
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>30</v>
+        <v>431</v>
       </c>
       <c r="B48" t="s">
-        <v>384</v>
+        <v>447</v>
       </c>
       <c r="C48" t="s">
-        <v>236</v>
-      </c>
-      <c r="E48" t="s">
-        <v>430</v>
+        <v>235</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>202</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>437</v>
+        <v>30</v>
       </c>
       <c r="B49" t="s">
-        <v>456</v>
+        <v>384</v>
       </c>
       <c r="C49" t="s">
         <v>236</v>
       </c>
-      <c r="D49" s="2" t="s">
-        <v>202</v>
+      <c r="E49" t="s">
+        <v>430</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="B50" t="s">
-        <v>448</v>
+        <v>456</v>
       </c>
       <c r="C50" t="s">
         <v>236</v>
@@ -2498,35 +2498,32 @@
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>95</v>
+        <v>438</v>
       </c>
       <c r="B51" t="s">
-        <v>368</v>
-      </c>
-      <c r="E51" t="s">
-        <v>396</v>
+        <v>448</v>
+      </c>
+      <c r="C51" t="s">
+        <v>236</v>
+      </c>
+      <c r="D51" s="2" t="s">
+        <v>202</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>31</v>
+        <v>95</v>
       </c>
       <c r="B52" t="s">
-        <v>237</v>
-      </c>
-      <c r="C52" s="3" t="s">
-        <v>238</v>
-      </c>
-      <c r="D52" s="3" t="s">
-        <v>239</v>
+        <v>368</v>
       </c>
       <c r="E52" t="s">
-        <v>430</v>
+        <v>396</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>97</v>
+        <v>31</v>
       </c>
       <c r="B53" t="s">
         <v>237</v>
@@ -2537,27 +2534,30 @@
       <c r="D53" s="3" t="s">
         <v>239</v>
       </c>
+      <c r="E53" t="s">
+        <v>430</v>
+      </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>439</v>
+        <v>97</v>
       </c>
       <c r="B54" t="s">
-        <v>457</v>
+        <v>237</v>
       </c>
       <c r="C54" s="3" t="s">
         <v>238</v>
       </c>
-      <c r="D54" s="2" t="s">
-        <v>202</v>
+      <c r="D54" s="3" t="s">
+        <v>239</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>432</v>
+        <v>439</v>
       </c>
       <c r="B55" t="s">
-        <v>449</v>
+        <v>457</v>
       </c>
       <c r="C55" s="3" t="s">
         <v>238</v>
@@ -2568,41 +2568,41 @@
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>32</v>
+        <v>432</v>
       </c>
       <c r="B56" t="s">
-        <v>240</v>
-      </c>
-      <c r="C56" t="s">
+        <v>449</v>
+      </c>
+      <c r="C56" s="3" t="s">
         <v>238</v>
       </c>
-      <c r="D56" t="s">
-        <v>223</v>
-      </c>
-      <c r="E56" t="s">
-        <v>430</v>
+      <c r="D56" s="2" t="s">
+        <v>202</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>440</v>
+        <v>32</v>
       </c>
       <c r="B57" t="s">
-        <v>458</v>
+        <v>240</v>
       </c>
       <c r="C57" t="s">
         <v>238</v>
       </c>
-      <c r="D57" s="2" t="s">
-        <v>202</v>
+      <c r="D57" t="s">
+        <v>223</v>
+      </c>
+      <c r="E57" t="s">
+        <v>430</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>433</v>
+        <v>440</v>
       </c>
       <c r="B58" t="s">
-        <v>450</v>
+        <v>458</v>
       </c>
       <c r="C58" t="s">
         <v>238</v>
@@ -2613,39 +2613,39 @@
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>33</v>
+        <v>433</v>
       </c>
       <c r="B59" t="s">
-        <v>241</v>
-      </c>
-      <c r="C59" s="3" t="s">
-        <v>242</v>
-      </c>
-      <c r="D59" s="3"/>
-      <c r="E59" t="s">
-        <v>430</v>
+        <v>450</v>
+      </c>
+      <c r="C59" t="s">
+        <v>238</v>
+      </c>
+      <c r="D59" s="2" t="s">
+        <v>202</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>441</v>
+        <v>33</v>
       </c>
       <c r="B60" t="s">
-        <v>459</v>
+        <v>241</v>
       </c>
       <c r="C60" s="3" t="s">
         <v>242</v>
       </c>
-      <c r="D60" s="2" t="s">
-        <v>202</v>
+      <c r="D60" s="3"/>
+      <c r="E60" t="s">
+        <v>430</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>434</v>
+        <v>441</v>
       </c>
       <c r="B61" t="s">
-        <v>451</v>
+        <v>459</v>
       </c>
       <c r="C61" s="3" t="s">
         <v>242</v>
@@ -2656,21 +2656,21 @@
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>34</v>
+        <v>434</v>
       </c>
       <c r="B62" t="s">
-        <v>397</v>
-      </c>
-      <c r="C62" t="s">
-        <v>243</v>
-      </c>
-      <c r="E62" t="s">
-        <v>398</v>
+        <v>451</v>
+      </c>
+      <c r="C62" s="3" t="s">
+        <v>242</v>
+      </c>
+      <c r="D62" s="2" t="s">
+        <v>202</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>101</v>
+        <v>34</v>
       </c>
       <c r="B63" t="s">
         <v>397</v>
@@ -2684,39 +2684,39 @@
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>35</v>
+        <v>101</v>
       </c>
       <c r="B64" t="s">
-        <v>244</v>
-      </c>
-      <c r="C64" s="3" t="s">
-        <v>463</v>
-      </c>
-      <c r="D64" s="3"/>
+        <v>397</v>
+      </c>
+      <c r="C64" t="s">
+        <v>243</v>
+      </c>
       <c r="E64" t="s">
-        <v>430</v>
+        <v>398</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>442</v>
+        <v>35</v>
       </c>
       <c r="B65" t="s">
-        <v>460</v>
+        <v>244</v>
       </c>
       <c r="C65" s="3" t="s">
         <v>463</v>
       </c>
-      <c r="D65" s="2" t="s">
-        <v>202</v>
+      <c r="D65" s="3"/>
+      <c r="E65" t="s">
+        <v>430</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>435</v>
+        <v>442</v>
       </c>
       <c r="B66" t="s">
-        <v>452</v>
+        <v>460</v>
       </c>
       <c r="C66" s="3" t="s">
         <v>463</v>
@@ -2727,38 +2727,38 @@
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>36</v>
+        <v>435</v>
       </c>
       <c r="B67" t="s">
-        <v>245</v>
+        <v>452</v>
       </c>
       <c r="C67" s="3" t="s">
         <v>463</v>
       </c>
+      <c r="D67" s="2" t="s">
+        <v>202</v>
+      </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B68" t="s">
-        <v>462</v>
-      </c>
-      <c r="C68" t="s">
-        <v>201</v>
-      </c>
-      <c r="D68" t="s">
-        <v>202</v>
+        <v>245</v>
+      </c>
+      <c r="C68" s="3" t="s">
+        <v>463</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B69" t="s">
-        <v>246</v>
-      </c>
-      <c r="C69" s="4" t="s">
-        <v>464</v>
+        <v>462</v>
+      </c>
+      <c r="C69" t="s">
+        <v>201</v>
       </c>
       <c r="D69" t="s">
         <v>202</v>
@@ -2766,46 +2766,49 @@
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B70" t="s">
-        <v>247</v>
-      </c>
-      <c r="C70" t="s">
-        <v>248</v>
+        <v>246</v>
+      </c>
+      <c r="C70" s="4" t="s">
+        <v>464</v>
       </c>
       <c r="D70" t="s">
-        <v>249</v>
+        <v>202</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B71" t="s">
-        <v>250</v>
+        <v>247</v>
+      </c>
+      <c r="C71" t="s">
+        <v>248</v>
       </c>
       <c r="D71" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B72" t="s">
-        <v>373</v>
-      </c>
-      <c r="D72" s="2" t="s">
-        <v>202</v>
+        <v>250</v>
+      </c>
+      <c r="D72" t="s">
+        <v>251</v>
       </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B73" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="D73" s="2" t="s">
         <v>202</v>
@@ -2813,107 +2816,107 @@
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B74" t="s">
-        <v>282</v>
-      </c>
-      <c r="D74" t="s">
-        <v>266</v>
-      </c>
-      <c r="E74" t="s">
-        <v>283</v>
+        <v>374</v>
+      </c>
+      <c r="D74" s="2" t="s">
+        <v>202</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B75" t="s">
-        <v>284</v>
-      </c>
-      <c r="C75" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="D75" t="s">
         <v>266</v>
       </c>
       <c r="E75" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B76" t="s">
-        <v>375</v>
+        <v>284</v>
+      </c>
+      <c r="C76" t="s">
+        <v>285</v>
       </c>
       <c r="D76" t="s">
         <v>266</v>
       </c>
       <c r="E76" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B77" t="s">
-        <v>376</v>
+        <v>375</v>
+      </c>
+      <c r="D77" t="s">
+        <v>266</v>
+      </c>
+      <c r="E77" t="s">
+        <v>287</v>
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B78" t="s">
-        <v>252</v>
+        <v>376</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B79" t="s">
-        <v>253</v>
-      </c>
-      <c r="D79" t="s">
-        <v>223</v>
+        <v>252</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B80" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="D80" t="s">
-        <v>202</v>
+        <v>223</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B81" t="s">
-        <v>255</v>
-      </c>
-      <c r="C81" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="D81" t="s">
-        <v>223</v>
+        <v>202</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B82" t="s">
-        <v>257</v>
+        <v>255</v>
+      </c>
+      <c r="C82" t="s">
+        <v>256</v>
       </c>
       <c r="D82" t="s">
         <v>223</v>
@@ -2921,85 +2924,81 @@
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B83" t="s">
-        <v>258</v>
+        <v>257</v>
+      </c>
+      <c r="D83" t="s">
+        <v>223</v>
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B84" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B85" t="s">
-        <v>260</v>
-      </c>
-      <c r="C85" t="s">
-        <v>256</v>
-      </c>
-      <c r="E85" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B86" t="s">
-        <v>262</v>
+        <v>260</v>
+      </c>
+      <c r="C86" t="s">
+        <v>256</v>
+      </c>
+      <c r="E86" t="s">
+        <v>261</v>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B87" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B88" t="s">
-        <v>264</v>
-      </c>
-      <c r="C88" t="s">
-        <v>256</v>
-      </c>
-      <c r="E88" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B89" t="s">
-        <v>265</v>
-      </c>
-      <c r="D89" s="2" t="s">
-        <v>266</v>
-      </c>
-      <c r="E89" s="1"/>
+        <v>264</v>
+      </c>
+      <c r="C89" t="s">
+        <v>256</v>
+      </c>
+      <c r="E89" t="s">
+        <v>261</v>
+      </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B90" t="s">
-        <v>267</v>
-      </c>
-      <c r="C90" t="s">
-        <v>256</v>
+        <v>265</v>
       </c>
       <c r="D90" s="2" t="s">
         <v>266</v>
@@ -3008,138 +3007,142 @@
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B91" t="s">
-        <v>268</v>
-      </c>
+        <v>267</v>
+      </c>
+      <c r="C91" t="s">
+        <v>256</v>
+      </c>
+      <c r="D91" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="E91" s="1"/>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B92" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B93" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B94" t="s">
-        <v>271</v>
-      </c>
-      <c r="C94" t="s">
-        <v>256</v>
-      </c>
-      <c r="E94" t="s">
-        <v>261</v>
+        <v>270</v>
       </c>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B95" t="s">
-        <v>272</v>
+        <v>271</v>
+      </c>
+      <c r="C95" t="s">
+        <v>256</v>
+      </c>
+      <c r="E95" t="s">
+        <v>261</v>
       </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B96" t="s">
-        <v>273</v>
-      </c>
-      <c r="D96" s="5" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B97" t="s">
-        <v>275</v>
-      </c>
-      <c r="C97" t="s">
-        <v>256</v>
+        <v>273</v>
       </c>
       <c r="D97" s="5" t="s">
         <v>274</v>
       </c>
-      <c r="E97" t="s">
-        <v>261</v>
-      </c>
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B98" t="s">
-        <v>276</v>
+        <v>275</v>
+      </c>
+      <c r="C98" t="s">
+        <v>256</v>
+      </c>
+      <c r="D98" s="5" t="s">
+        <v>274</v>
+      </c>
+      <c r="E98" t="s">
+        <v>261</v>
       </c>
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>68</v>
-      </c>
-      <c r="B99" s="6" t="s">
-        <v>277</v>
+        <v>67</v>
+      </c>
+      <c r="B99" t="s">
+        <v>276</v>
       </c>
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B100" s="6" t="s">
-        <v>278</v>
-      </c>
-      <c r="E100" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="101" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>70</v>
-      </c>
-      <c r="B101" t="s">
-        <v>280</v>
+        <v>69</v>
+      </c>
+      <c r="B101" s="6" t="s">
+        <v>278</v>
+      </c>
+      <c r="E101" t="s">
+        <v>279</v>
       </c>
     </row>
     <row r="102" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B102" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B103" t="s">
-        <v>377</v>
-      </c>
-      <c r="D103" t="s">
-        <v>380</v>
+        <v>281</v>
       </c>
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B104" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="D104" t="s">
         <v>380</v>
@@ -3147,13 +3150,10 @@
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B105" t="s">
-        <v>378</v>
-      </c>
-      <c r="C105" t="s">
-        <v>256</v>
+        <v>379</v>
       </c>
       <c r="D105" t="s">
         <v>380</v>
@@ -3161,26 +3161,32 @@
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B106" t="s">
-        <v>381</v>
+        <v>378</v>
+      </c>
+      <c r="C106" t="s">
+        <v>256</v>
       </c>
       <c r="D106" t="s">
-        <v>202</v>
+        <v>380</v>
       </c>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B107" t="s">
-        <v>288</v>
+        <v>381</v>
+      </c>
+      <c r="D107" t="s">
+        <v>202</v>
       </c>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>99</v>
+        <v>76</v>
       </c>
       <c r="B108" t="s">
         <v>288</v>
@@ -3188,91 +3194,88 @@
     </row>
     <row r="109" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>77</v>
+        <v>99</v>
       </c>
       <c r="B109" t="s">
-        <v>289</v>
-      </c>
-      <c r="D109" t="s">
-        <v>290</v>
-      </c>
-      <c r="E109" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
     </row>
     <row r="110" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B110" t="s">
-        <v>292</v>
-      </c>
-      <c r="D110" s="2" t="s">
-        <v>293</v>
+        <v>289</v>
+      </c>
+      <c r="D110" t="s">
+        <v>290</v>
       </c>
       <c r="E110" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
     </row>
     <row r="111" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B111" t="s">
         <v>292</v>
       </c>
       <c r="D111" s="2" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="E111" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
     </row>
     <row r="112" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B112" t="s">
-        <v>297</v>
+        <v>292</v>
       </c>
       <c r="D112" s="2" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="E112" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
     </row>
     <row r="113" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B113" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="D113" s="2" t="s">
         <v>293</v>
       </c>
       <c r="E113" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
     </row>
     <row r="114" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B114" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="D114" s="2" t="s">
         <v>293</v>
       </c>
+      <c r="E114" t="s">
+        <v>300</v>
+      </c>
     </row>
     <row r="115" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B115" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="D115" s="2" t="s">
         <v>293</v>
@@ -3280,38 +3283,35 @@
     </row>
     <row r="116" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B116" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="D116" s="2" t="s">
         <v>293</v>
       </c>
-      <c r="E116" t="s">
-        <v>304</v>
-      </c>
     </row>
     <row r="117" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B117" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="D117" s="2" t="s">
         <v>293</v>
       </c>
       <c r="E117" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
     </row>
     <row r="118" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B118" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="D118" s="2" t="s">
         <v>293</v>
@@ -3322,34 +3322,40 @@
     </row>
     <row r="119" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B119" t="s">
-        <v>308</v>
+        <v>307</v>
+      </c>
+      <c r="D119" s="2" t="s">
+        <v>293</v>
       </c>
       <c r="E119" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
     </row>
     <row r="120" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B120" t="s">
-        <v>310</v>
+        <v>308</v>
+      </c>
+      <c r="E120" t="s">
+        <v>309</v>
       </c>
     </row>
     <row r="121" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B121" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
     </row>
     <row r="122" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>107</v>
+        <v>89</v>
       </c>
       <c r="B122" t="s">
         <v>311</v>
@@ -3357,37 +3363,34 @@
     </row>
     <row r="123" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
-        <v>90</v>
+        <v>107</v>
       </c>
       <c r="B123" t="s">
-        <v>468</v>
+        <v>311</v>
       </c>
     </row>
     <row r="124" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
-        <v>399</v>
+        <v>90</v>
       </c>
       <c r="B124" t="s">
         <v>468</v>
       </c>
     </row>
     <row r="125" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A125" s="7" t="s">
-        <v>409</v>
+      <c r="A125" t="s">
+        <v>399</v>
       </c>
       <c r="B125" t="s">
-        <v>416</v>
-      </c>
-      <c r="D125" t="s">
-        <v>423</v>
+        <v>468</v>
       </c>
     </row>
     <row r="126" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A126" s="7" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="B126" t="s">
-        <v>419</v>
+        <v>416</v>
       </c>
       <c r="D126" t="s">
         <v>423</v>
@@ -3395,10 +3398,10 @@
     </row>
     <row r="127" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A127" s="7" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="B127" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="D127" t="s">
         <v>423</v>
@@ -3406,10 +3409,10 @@
     </row>
     <row r="128" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A128" s="7" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="B128" t="s">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="D128" t="s">
         <v>423</v>
@@ -3417,10 +3420,10 @@
     </row>
     <row r="129" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A129" s="7" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="B129" t="s">
-        <v>421</v>
+        <v>417</v>
       </c>
       <c r="D129" t="s">
         <v>423</v>
@@ -3428,10 +3431,10 @@
     </row>
     <row r="130" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A130" s="7" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="B130" t="s">
-        <v>418</v>
+        <v>421</v>
       </c>
       <c r="D130" t="s">
         <v>423</v>
@@ -3439,32 +3442,29 @@
     </row>
     <row r="131" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A131" s="7" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="B131" t="s">
-        <v>422</v>
+        <v>418</v>
       </c>
       <c r="D131" t="s">
         <v>423</v>
       </c>
     </row>
     <row r="132" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A132" t="s">
-        <v>91</v>
+      <c r="A132" s="7" t="s">
+        <v>415</v>
       </c>
       <c r="B132" t="s">
-        <v>312</v>
-      </c>
-      <c r="C132" t="s">
-        <v>313</v>
-      </c>
-      <c r="E132" t="s">
-        <v>314</v>
+        <v>422</v>
+      </c>
+      <c r="D132" t="s">
+        <v>423</v>
       </c>
     </row>
     <row r="133" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="B133" t="s">
         <v>312</v>
@@ -3472,24 +3472,24 @@
       <c r="C133" t="s">
         <v>313</v>
       </c>
+      <c r="E133" t="s">
+        <v>314</v>
+      </c>
     </row>
     <row r="134" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
-        <v>479</v>
+        <v>100</v>
       </c>
       <c r="B134" t="s">
-        <v>491</v>
+        <v>312</v>
       </c>
       <c r="C134" t="s">
-        <v>201</v>
-      </c>
-      <c r="E134" t="s">
-        <v>497</v>
+        <v>313</v>
       </c>
     </row>
     <row r="135" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="B135" t="s">
         <v>491</v>
@@ -3503,10 +3503,10 @@
     </row>
     <row r="136" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="B136" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="C136" t="s">
         <v>201</v>
@@ -3517,7 +3517,7 @@
     </row>
     <row r="137" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="B137" t="s">
         <v>492</v>
@@ -3531,10 +3531,10 @@
     </row>
     <row r="138" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="B138" t="s">
-        <v>494</v>
+        <v>492</v>
       </c>
       <c r="C138" t="s">
         <v>201</v>
@@ -3545,7 +3545,7 @@
     </row>
     <row r="139" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="B139" t="s">
         <v>494</v>
@@ -3559,10 +3559,10 @@
     </row>
     <row r="140" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="B140" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="C140" t="s">
         <v>201</v>
@@ -3573,7 +3573,7 @@
     </row>
     <row r="141" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="B141" t="s">
         <v>493</v>
@@ -3587,10 +3587,10 @@
     </row>
     <row r="142" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="B142" t="s">
-        <v>495</v>
+        <v>493</v>
       </c>
       <c r="C142" t="s">
         <v>201</v>
@@ -3601,7 +3601,7 @@
     </row>
     <row r="143" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="B143" t="s">
         <v>495</v>
@@ -3615,10 +3615,10 @@
     </row>
     <row r="144" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="B144" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="C144" t="s">
         <v>201</v>
@@ -3629,7 +3629,7 @@
     </row>
     <row r="145" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="B145" t="s">
         <v>496</v>
@@ -3638,212 +3638,215 @@
         <v>201</v>
       </c>
       <c r="E145" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
     </row>
     <row r="146" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
-        <v>400</v>
+        <v>490</v>
       </c>
       <c r="B146" t="s">
-        <v>401</v>
+        <v>496</v>
+      </c>
+      <c r="C146" t="s">
+        <v>201</v>
       </c>
       <c r="E146" t="s">
-        <v>402</v>
+        <v>498</v>
       </c>
     </row>
     <row r="147" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
-        <v>102</v>
+        <v>400</v>
       </c>
       <c r="B147" t="s">
-        <v>299</v>
-      </c>
-      <c r="C147" s="3"/>
+        <v>401</v>
+      </c>
       <c r="E147" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
     </row>
     <row r="148" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B148" t="s">
-        <v>369</v>
-      </c>
+        <v>299</v>
+      </c>
+      <c r="C148" s="3"/>
       <c r="E148" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="149" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B149" t="s">
-        <v>297</v>
-      </c>
-      <c r="C149" s="3"/>
+        <v>369</v>
+      </c>
       <c r="E149" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="150" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B150" t="s">
-        <v>292</v>
-      </c>
+        <v>297</v>
+      </c>
+      <c r="C150" s="3"/>
       <c r="E150" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="151" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B151" t="s">
-        <v>302</v>
+        <v>292</v>
       </c>
       <c r="E151" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
     </row>
     <row r="152" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B152" t="s">
-        <v>315</v>
+        <v>302</v>
+      </c>
+      <c r="E152" t="s">
+        <v>407</v>
       </c>
     </row>
     <row r="153" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B153" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="154" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B154" t="s">
-        <v>465</v>
-      </c>
-      <c r="E154" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
     </row>
     <row r="155" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B155" t="s">
-        <v>318</v>
+        <v>465</v>
       </c>
       <c r="E155" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
     </row>
     <row r="156" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B156" t="s">
-        <v>320</v>
-      </c>
-      <c r="C156" t="s">
-        <v>321</v>
+        <v>318</v>
+      </c>
+      <c r="E156" t="s">
+        <v>319</v>
       </c>
     </row>
     <row r="157" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B157" t="s">
-        <v>322</v>
+        <v>320</v>
+      </c>
+      <c r="C157" t="s">
+        <v>321</v>
       </c>
     </row>
     <row r="158" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B158" t="s">
-        <v>219</v>
-      </c>
-      <c r="C158" t="s">
-        <v>197</v>
-      </c>
-      <c r="E158" t="s">
-        <v>499</v>
+        <v>322</v>
       </c>
     </row>
     <row r="159" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
-        <v>389</v>
+        <v>114</v>
       </c>
       <c r="B159" t="s">
-        <v>323</v>
+        <v>219</v>
       </c>
       <c r="C159" t="s">
         <v>197</v>
       </c>
       <c r="E159" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
     </row>
     <row r="160" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
-        <v>115</v>
+        <v>389</v>
       </c>
       <c r="B160" t="s">
-        <v>213</v>
+        <v>323</v>
+      </c>
+      <c r="C160" t="s">
+        <v>197</v>
       </c>
       <c r="E160" t="s">
-        <v>324</v>
+        <v>500</v>
       </c>
     </row>
     <row r="161" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B161" t="s">
-        <v>297</v>
+        <v>213</v>
       </c>
       <c r="E161" t="s">
-        <v>501</v>
+        <v>324</v>
       </c>
     </row>
     <row r="162" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B162" t="s">
-        <v>292</v>
+        <v>297</v>
       </c>
       <c r="E162" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
     </row>
     <row r="163" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B163" t="s">
-        <v>325</v>
+        <v>292</v>
       </c>
       <c r="E163" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
     </row>
     <row r="164" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B164" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="E164" t="s">
         <v>503</v>
@@ -3851,10 +3854,10 @@
     </row>
     <row r="165" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B165" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="E165" t="s">
         <v>503</v>
@@ -3862,10 +3865,10 @@
     </row>
     <row r="166" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B166" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="E166" t="s">
         <v>503</v>
@@ -3873,10 +3876,10 @@
     </row>
     <row r="167" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B167" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="E167" t="s">
         <v>503</v>
@@ -3884,54 +3887,54 @@
     </row>
     <row r="168" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B168" t="s">
-        <v>303</v>
+        <v>329</v>
       </c>
       <c r="E168" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
     </row>
     <row r="169" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B169" t="s">
-        <v>330</v>
+        <v>303</v>
       </c>
       <c r="E169" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
     </row>
     <row r="170" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B170" t="s">
-        <v>299</v>
+        <v>330</v>
       </c>
       <c r="E170" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
     </row>
     <row r="171" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B171" t="s">
-        <v>331</v>
+        <v>299</v>
       </c>
       <c r="E171" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
     </row>
     <row r="172" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B172" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="E172" t="s">
         <v>503</v>
@@ -3939,10 +3942,10 @@
     </row>
     <row r="173" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B173" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="E173" t="s">
         <v>503</v>
@@ -3950,10 +3953,10 @@
     </row>
     <row r="174" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B174" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="E174" t="s">
         <v>503</v>
@@ -3961,10 +3964,10 @@
     </row>
     <row r="175" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
-        <v>385</v>
+        <v>129</v>
       </c>
       <c r="B175" t="s">
-        <v>386</v>
+        <v>334</v>
       </c>
       <c r="E175" t="s">
         <v>503</v>
@@ -3972,10 +3975,10 @@
     </row>
     <row r="176" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
-        <v>130</v>
+        <v>385</v>
       </c>
       <c r="B176" t="s">
-        <v>335</v>
+        <v>386</v>
       </c>
       <c r="E176" t="s">
         <v>503</v>
@@ -3983,10 +3986,10 @@
     </row>
     <row r="177" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B177" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="E177" t="s">
         <v>503</v>
@@ -3994,10 +3997,10 @@
     </row>
     <row r="178" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B178" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="E178" t="s">
         <v>503</v>
@@ -4005,10 +4008,10 @@
     </row>
     <row r="179" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B179" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="E179" t="s">
         <v>503</v>
@@ -4016,10 +4019,10 @@
     </row>
     <row r="180" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
-        <v>387</v>
+        <v>133</v>
       </c>
       <c r="B180" t="s">
-        <v>388</v>
+        <v>338</v>
       </c>
       <c r="E180" t="s">
         <v>503</v>
@@ -4027,10 +4030,10 @@
     </row>
     <row r="181" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
-        <v>134</v>
+        <v>387</v>
       </c>
       <c r="B181" t="s">
-        <v>339</v>
+        <v>388</v>
       </c>
       <c r="E181" t="s">
         <v>503</v>
@@ -4038,10 +4041,10 @@
     </row>
     <row r="182" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B182" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="E182" t="s">
         <v>503</v>
@@ -4049,10 +4052,10 @@
     </row>
     <row r="183" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B183" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="E183" t="s">
         <v>503</v>
@@ -4060,10 +4063,10 @@
     </row>
     <row r="184" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B184" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="E184" t="s">
         <v>503</v>
@@ -4071,10 +4074,10 @@
     </row>
     <row r="185" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B185" t="s">
-        <v>475</v>
+        <v>342</v>
       </c>
       <c r="E185" t="s">
         <v>503</v>
@@ -4082,10 +4085,10 @@
     </row>
     <row r="186" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B186" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="E186" t="s">
         <v>503</v>
@@ -4093,10 +4096,10 @@
     </row>
     <row r="187" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B187" t="s">
-        <v>343</v>
+        <v>476</v>
       </c>
       <c r="E187" t="s">
         <v>503</v>
@@ -4104,10 +4107,10 @@
     </row>
     <row r="188" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A188" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B188" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="E188" t="s">
         <v>503</v>
@@ -4115,10 +4118,10 @@
     </row>
     <row r="189" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B189" t="s">
-        <v>390</v>
+        <v>344</v>
       </c>
       <c r="E189" t="s">
         <v>503</v>
@@ -4126,7 +4129,7 @@
     </row>
     <row r="190" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
-        <v>408</v>
+        <v>142</v>
       </c>
       <c r="B190" t="s">
         <v>390</v>
@@ -4137,10 +4140,10 @@
     </row>
     <row r="191" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
-        <v>466</v>
+        <v>408</v>
       </c>
       <c r="B191" t="s">
-        <v>467</v>
+        <v>390</v>
       </c>
       <c r="E191" t="s">
         <v>503</v>
@@ -4148,10 +4151,10 @@
     </row>
     <row r="192" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
-        <v>143</v>
+        <v>466</v>
       </c>
       <c r="B192" t="s">
-        <v>345</v>
+        <v>467</v>
       </c>
       <c r="E192" t="s">
         <v>503</v>
@@ -4159,10 +4162,10 @@
     </row>
     <row r="193" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
-        <v>144</v>
-      </c>
-      <c r="C193" t="s">
-        <v>197</v>
+        <v>143</v>
+      </c>
+      <c r="B193" t="s">
+        <v>345</v>
       </c>
       <c r="E193" t="s">
         <v>503</v>
@@ -4170,10 +4173,10 @@
     </row>
     <row r="194" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A194" t="s">
-        <v>145</v>
-      </c>
-      <c r="B194" t="s">
-        <v>346</v>
+        <v>144</v>
+      </c>
+      <c r="C194" t="s">
+        <v>197</v>
       </c>
       <c r="E194" t="s">
         <v>503</v>
@@ -4181,10 +4184,10 @@
     </row>
     <row r="195" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B195" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="E195" t="s">
         <v>503</v>
@@ -4192,10 +4195,10 @@
     </row>
     <row r="196" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A196" t="s">
-        <v>147</v>
-      </c>
-      <c r="C196" t="s">
-        <v>197</v>
+        <v>146</v>
+      </c>
+      <c r="B196" t="s">
+        <v>347</v>
       </c>
       <c r="E196" t="s">
         <v>503</v>
@@ -4203,10 +4206,10 @@
     </row>
     <row r="197" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
-        <v>148</v>
-      </c>
-      <c r="B197" t="s">
-        <v>348</v>
+        <v>147</v>
+      </c>
+      <c r="C197" t="s">
+        <v>197</v>
       </c>
       <c r="E197" t="s">
         <v>503</v>
@@ -4214,10 +4217,10 @@
     </row>
     <row r="198" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A198" t="s">
-        <v>149</v>
-      </c>
-      <c r="C198" t="s">
-        <v>197</v>
+        <v>148</v>
+      </c>
+      <c r="B198" t="s">
+        <v>348</v>
       </c>
       <c r="E198" t="s">
         <v>503</v>
@@ -4225,10 +4228,10 @@
     </row>
     <row r="199" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A199" t="s">
-        <v>150</v>
-      </c>
-      <c r="B199" t="s">
-        <v>349</v>
+        <v>149</v>
+      </c>
+      <c r="C199" t="s">
+        <v>197</v>
       </c>
       <c r="E199" t="s">
         <v>503</v>
@@ -4236,10 +4239,10 @@
     </row>
     <row r="200" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A200" t="s">
-        <v>151</v>
-      </c>
-      <c r="C200" t="s">
-        <v>197</v>
+        <v>150</v>
+      </c>
+      <c r="B200" t="s">
+        <v>349</v>
       </c>
       <c r="E200" t="s">
         <v>503</v>
@@ -4247,10 +4250,10 @@
     </row>
     <row r="201" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A201" t="s">
-        <v>152</v>
-      </c>
-      <c r="B201" t="s">
-        <v>350</v>
+        <v>151</v>
+      </c>
+      <c r="C201" t="s">
+        <v>197</v>
       </c>
       <c r="E201" t="s">
         <v>503</v>
@@ -4258,10 +4261,10 @@
     </row>
     <row r="202" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A202" t="s">
-        <v>153</v>
-      </c>
-      <c r="C202" t="s">
-        <v>197</v>
+        <v>152</v>
+      </c>
+      <c r="B202" t="s">
+        <v>350</v>
       </c>
       <c r="E202" t="s">
         <v>503</v>
@@ -4269,10 +4272,10 @@
     </row>
     <row r="203" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A203" t="s">
-        <v>154</v>
-      </c>
-      <c r="B203" t="s">
-        <v>351</v>
+        <v>153</v>
+      </c>
+      <c r="C203" t="s">
+        <v>197</v>
       </c>
       <c r="E203" t="s">
         <v>503</v>
@@ -4280,10 +4283,10 @@
     </row>
     <row r="204" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A204" t="s">
-        <v>155</v>
-      </c>
-      <c r="C204" t="s">
-        <v>197</v>
+        <v>154</v>
+      </c>
+      <c r="B204" t="s">
+        <v>351</v>
       </c>
       <c r="E204" t="s">
         <v>503</v>
@@ -4291,10 +4294,10 @@
     </row>
     <row r="205" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A205" t="s">
-        <v>156</v>
-      </c>
-      <c r="B205" t="s">
-        <v>352</v>
+        <v>155</v>
+      </c>
+      <c r="C205" t="s">
+        <v>197</v>
       </c>
       <c r="E205" t="s">
         <v>503</v>
@@ -4302,10 +4305,10 @@
     </row>
     <row r="206" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A206" t="s">
-        <v>157</v>
-      </c>
-      <c r="C206" t="s">
-        <v>197</v>
+        <v>156</v>
+      </c>
+      <c r="B206" t="s">
+        <v>352</v>
       </c>
       <c r="E206" t="s">
         <v>503</v>
@@ -4313,10 +4316,10 @@
     </row>
     <row r="207" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
-        <v>158</v>
-      </c>
-      <c r="B207" t="s">
-        <v>353</v>
+        <v>157</v>
+      </c>
+      <c r="C207" t="s">
+        <v>197</v>
       </c>
       <c r="E207" t="s">
         <v>503</v>
@@ -4324,10 +4327,10 @@
     </row>
     <row r="208" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A208" t="s">
-        <v>159</v>
-      </c>
-      <c r="C208" t="s">
-        <v>197</v>
+        <v>158</v>
+      </c>
+      <c r="B208" t="s">
+        <v>353</v>
       </c>
       <c r="E208" t="s">
         <v>503</v>
@@ -4335,7 +4338,7 @@
     </row>
     <row r="209" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A209" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C209" t="s">
         <v>197</v>
@@ -4346,10 +4349,10 @@
     </row>
     <row r="210" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A210" t="s">
-        <v>161</v>
-      </c>
-      <c r="B210" t="s">
-        <v>354</v>
+        <v>160</v>
+      </c>
+      <c r="C210" t="s">
+        <v>197</v>
       </c>
       <c r="E210" t="s">
         <v>503</v>
@@ -4357,10 +4360,10 @@
     </row>
     <row r="211" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A211" t="s">
-        <v>162</v>
-      </c>
-      <c r="C211" t="s">
-        <v>197</v>
+        <v>161</v>
+      </c>
+      <c r="B211" t="s">
+        <v>354</v>
       </c>
       <c r="E211" t="s">
         <v>503</v>
@@ -4368,10 +4371,10 @@
     </row>
     <row r="212" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A212" t="s">
-        <v>163</v>
-      </c>
-      <c r="B212" t="s">
-        <v>355</v>
+        <v>162</v>
+      </c>
+      <c r="C212" t="s">
+        <v>197</v>
       </c>
       <c r="E212" t="s">
         <v>503</v>
@@ -4379,10 +4382,10 @@
     </row>
     <row r="213" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A213" t="s">
-        <v>164</v>
-      </c>
-      <c r="C213" t="s">
-        <v>197</v>
+        <v>163</v>
+      </c>
+      <c r="B213" t="s">
+        <v>355</v>
       </c>
       <c r="E213" t="s">
         <v>503</v>
@@ -4390,10 +4393,10 @@
     </row>
     <row r="214" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A214" t="s">
-        <v>469</v>
-      </c>
-      <c r="B214" t="s">
-        <v>471</v>
+        <v>164</v>
+      </c>
+      <c r="C214" t="s">
+        <v>197</v>
       </c>
       <c r="E214" t="s">
         <v>503</v>
@@ -4401,21 +4404,21 @@
     </row>
     <row r="215" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
+        <v>469</v>
+      </c>
+      <c r="B215" t="s">
+        <v>471</v>
+      </c>
+      <c r="E215" t="s">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="216" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A216" t="s">
         <v>470</v>
       </c>
-      <c r="C215" t="s">
+      <c r="C216" t="s">
         <v>197</v>
-      </c>
-      <c r="E215" t="s">
-        <v>503</v>
-      </c>
-    </row>
-    <row r="216" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A216" s="7" t="s">
-        <v>472</v>
-      </c>
-      <c r="B216" t="s">
-        <v>474</v>
       </c>
       <c r="E216" t="s">
         <v>503</v>
@@ -4423,21 +4426,21 @@
     </row>
     <row r="217" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A217" s="7" t="s">
+        <v>472</v>
+      </c>
+      <c r="B217" t="s">
+        <v>474</v>
+      </c>
+      <c r="E217" t="s">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="218" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A218" s="7" t="s">
         <v>473</v>
       </c>
-      <c r="C217" t="s">
+      <c r="C218" t="s">
         <v>197</v>
-      </c>
-      <c r="E217" t="s">
-        <v>503</v>
-      </c>
-    </row>
-    <row r="218" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A218" t="s">
-        <v>165</v>
-      </c>
-      <c r="B218" t="s">
-        <v>356</v>
       </c>
       <c r="E218" t="s">
         <v>503</v>
@@ -4445,10 +4448,10 @@
     </row>
     <row r="219" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A219" t="s">
-        <v>166</v>
-      </c>
-      <c r="C219" t="s">
-        <v>197</v>
+        <v>165</v>
+      </c>
+      <c r="B219" t="s">
+        <v>356</v>
       </c>
       <c r="E219" t="s">
         <v>503</v>
@@ -4456,10 +4459,10 @@
     </row>
     <row r="220" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A220" t="s">
-        <v>167</v>
-      </c>
-      <c r="B220" t="s">
-        <v>357</v>
+        <v>166</v>
+      </c>
+      <c r="C220" t="s">
+        <v>197</v>
       </c>
       <c r="E220" t="s">
         <v>503</v>
@@ -4467,10 +4470,10 @@
     </row>
     <row r="221" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A221" t="s">
-        <v>168</v>
-      </c>
-      <c r="C221" t="s">
-        <v>197</v>
+        <v>167</v>
+      </c>
+      <c r="B221" t="s">
+        <v>357</v>
       </c>
       <c r="E221" t="s">
         <v>503</v>
@@ -4478,10 +4481,10 @@
     </row>
     <row r="222" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A222" t="s">
-        <v>169</v>
-      </c>
-      <c r="B222" t="s">
-        <v>358</v>
+        <v>168</v>
+      </c>
+      <c r="C222" t="s">
+        <v>197</v>
       </c>
       <c r="E222" t="s">
         <v>503</v>
@@ -4489,10 +4492,10 @@
     </row>
     <row r="223" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A223" t="s">
-        <v>170</v>
-      </c>
-      <c r="C223" t="s">
-        <v>197</v>
+        <v>169</v>
+      </c>
+      <c r="B223" t="s">
+        <v>358</v>
       </c>
       <c r="E223" t="s">
         <v>503</v>
@@ -4500,10 +4503,10 @@
     </row>
     <row r="224" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A224" t="s">
-        <v>171</v>
-      </c>
-      <c r="B224" t="s">
-        <v>359</v>
+        <v>170</v>
+      </c>
+      <c r="C224" t="s">
+        <v>197</v>
       </c>
       <c r="E224" t="s">
         <v>503</v>
@@ -4511,10 +4514,10 @@
     </row>
     <row r="225" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A225" t="s">
-        <v>172</v>
-      </c>
-      <c r="C225" t="s">
-        <v>197</v>
+        <v>171</v>
+      </c>
+      <c r="B225" t="s">
+        <v>359</v>
       </c>
       <c r="E225" t="s">
         <v>503</v>
@@ -4522,10 +4525,10 @@
     </row>
     <row r="226" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A226" t="s">
-        <v>173</v>
-      </c>
-      <c r="B226" t="s">
-        <v>360</v>
+        <v>172</v>
+      </c>
+      <c r="C226" t="s">
+        <v>197</v>
       </c>
       <c r="E226" t="s">
         <v>503</v>
@@ -4533,10 +4536,10 @@
     </row>
     <row r="227" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A227" t="s">
-        <v>174</v>
-      </c>
-      <c r="C227" t="s">
-        <v>197</v>
+        <v>173</v>
+      </c>
+      <c r="B227" t="s">
+        <v>360</v>
       </c>
       <c r="E227" t="s">
         <v>503</v>
@@ -4544,10 +4547,10 @@
     </row>
     <row r="228" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A228" t="s">
-        <v>175</v>
-      </c>
-      <c r="B228" t="s">
-        <v>361</v>
+        <v>174</v>
+      </c>
+      <c r="C228" t="s">
+        <v>197</v>
       </c>
       <c r="E228" t="s">
         <v>503</v>
@@ -4555,10 +4558,10 @@
     </row>
     <row r="229" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A229" t="s">
-        <v>176</v>
-      </c>
-      <c r="C229" t="s">
-        <v>197</v>
+        <v>175</v>
+      </c>
+      <c r="B229" t="s">
+        <v>361</v>
       </c>
       <c r="E229" t="s">
         <v>503</v>
@@ -4566,10 +4569,10 @@
     </row>
     <row r="230" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A230" t="s">
-        <v>177</v>
-      </c>
-      <c r="B230" t="s">
-        <v>362</v>
+        <v>176</v>
+      </c>
+      <c r="C230" t="s">
+        <v>197</v>
       </c>
       <c r="E230" t="s">
         <v>503</v>
@@ -4577,10 +4580,10 @@
     </row>
     <row r="231" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A231" t="s">
-        <v>178</v>
-      </c>
-      <c r="C231" t="s">
-        <v>197</v>
+        <v>177</v>
+      </c>
+      <c r="B231" t="s">
+        <v>362</v>
       </c>
       <c r="E231" t="s">
         <v>503</v>
@@ -4588,10 +4591,10 @@
     </row>
     <row r="232" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A232" t="s">
-        <v>179</v>
-      </c>
-      <c r="B232" t="s">
-        <v>363</v>
+        <v>178</v>
+      </c>
+      <c r="C232" t="s">
+        <v>197</v>
       </c>
       <c r="E232" t="s">
         <v>503</v>
@@ -4599,10 +4602,10 @@
     </row>
     <row r="233" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A233" t="s">
-        <v>180</v>
-      </c>
-      <c r="C233" t="s">
-        <v>197</v>
+        <v>179</v>
+      </c>
+      <c r="B233" t="s">
+        <v>363</v>
       </c>
       <c r="E233" t="s">
         <v>503</v>
@@ -4610,10 +4613,10 @@
     </row>
     <row r="234" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A234" t="s">
-        <v>181</v>
-      </c>
-      <c r="B234" t="s">
-        <v>364</v>
+        <v>180</v>
+      </c>
+      <c r="C234" t="s">
+        <v>197</v>
       </c>
       <c r="E234" t="s">
         <v>503</v>
@@ -4621,10 +4624,10 @@
     </row>
     <row r="235" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A235" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B235" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="E235" t="s">
         <v>503</v>
@@ -4632,10 +4635,10 @@
     </row>
     <row r="236" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A236" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B236" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="E236" t="s">
         <v>503</v>
@@ -4643,25 +4646,36 @@
     </row>
     <row r="237" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A237" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B237" t="s">
-        <v>382</v>
+        <v>366</v>
+      </c>
+      <c r="E237" t="s">
+        <v>503</v>
       </c>
     </row>
     <row r="238" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A238" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B238" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="239" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A239" t="s">
+        <v>185</v>
+      </c>
+      <c r="B239" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="240" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A240" t="s">
         <v>186</v>
       </c>
-      <c r="B239" t="s">
+      <c r="B240" t="s">
         <v>367</v>
       </c>
     </row>

</xml_diff>